<commit_message>
Chaîne régénérée de bout en bout au plafond 177 : figures, tables, HTML, PDF, docx, visualiseur
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/livrables/km_a_doubler.xlsx
+++ b/livrables/km_a_doubler.xlsx
@@ -438,7 +438,7 @@
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -527,7 +527,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Saint-Hyacinthe</t>
+          <t>Saint-Lambert</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">

</xml_diff>